<commit_message>
Se ectualizaron todos estos archivo
Sincronización atrasada
</commit_message>
<xml_diff>
--- a/layout/Credito_IFRS9_R04A_MOV_420_24.xlsx
+++ b/layout/Credito_IFRS9_R04A_MOV_420_24.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\LOCAL\DESA\non-purple-wheel\non-purple-wheel\layout\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78C0D648-0E73-4486-8395-92A56E8C6282}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D65D69DA-87EE-4BBF-B4F3-4222A2B03061}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="800" yWindow="2350" windowWidth="24380" windowHeight="17740" xr2:uid="{8DFCBC29-2A01-2140-94E8-D30E69B20726}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{8DFCBC29-2A01-2140-94E8-D30E69B20726}"/>
   </bookViews>
   <sheets>
     <sheet name="R04A_MOV_420_24" sheetId="2" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191028" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="50">
   <si>
     <t>LAYOUT</t>
   </si>
@@ -123,9 +123,6 @@
   </si>
   <si>
     <t>FECHA</t>
-  </si>
-  <si>
-    <t>8</t>
   </si>
   <si>
     <t>Debe ser una fecha valida</t>
@@ -674,23 +671,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B03CB0C2-A467-4E6E-8CC8-7C6AC6B12BBD}">
   <dimension ref="A1:P7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="19.33203125" customWidth="1"/>
-    <col min="2" max="2" width="5.58203125" customWidth="1"/>
-    <col min="3" max="3" width="8.33203125" customWidth="1"/>
-    <col min="4" max="4" width="22.33203125" customWidth="1"/>
-    <col min="5" max="5" width="11.58203125" customWidth="1"/>
-    <col min="6" max="6" width="11.33203125" customWidth="1"/>
+    <col min="1" max="1" width="19.375" customWidth="1"/>
+    <col min="2" max="2" width="5.625" customWidth="1"/>
+    <col min="3" max="3" width="8.375" customWidth="1"/>
+    <col min="4" max="4" width="22.375" customWidth="1"/>
+    <col min="5" max="5" width="11.625" customWidth="1"/>
+    <col min="6" max="6" width="11.375" customWidth="1"/>
     <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="24.33203125" customWidth="1"/>
-    <col min="9" max="9" width="26.33203125" customWidth="1"/>
-    <col min="10" max="10" width="9.33203125" customWidth="1"/>
-    <col min="11" max="11" width="24.58203125" customWidth="1"/>
-    <col min="12" max="12" width="56.58203125" customWidth="1"/>
-    <col min="13" max="13" width="29.83203125" customWidth="1"/>
+    <col min="8" max="8" width="24.375" customWidth="1"/>
+    <col min="9" max="9" width="26.375" customWidth="1"/>
+    <col min="10" max="10" width="9.375" customWidth="1"/>
+    <col min="11" max="11" width="24.625" customWidth="1"/>
+    <col min="12" max="12" width="56.625" customWidth="1"/>
+    <col min="13" max="13" width="29.875" customWidth="1"/>
     <col min="14" max="14" width="34" customWidth="1"/>
-    <col min="15" max="15" width="21.58203125" customWidth="1"/>
+    <col min="15" max="15" width="21.625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" s="1" customFormat="1">
@@ -745,7 +742,7 @@
     </row>
     <row r="2" spans="1:16">
       <c r="A2" s="8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B2" s="9">
         <v>1</v>
@@ -766,17 +763,17 @@
         <v>20</v>
       </c>
       <c r="H2" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="I2" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="J2" s="9" t="s">
         <v>34</v>
-      </c>
-      <c r="I2" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="J2" s="9" t="s">
-        <v>35</v>
       </c>
       <c r="K2" s="9"/>
       <c r="L2" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="M2" s="9" t="s">
         <v>21</v>
@@ -787,7 +784,7 @@
     </row>
     <row r="3" spans="1:16">
       <c r="A3" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B3" s="12">
         <v>2</v>
@@ -796,7 +793,7 @@
         <v>20</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E3" s="12" t="s">
         <v>23</v>
@@ -808,20 +805,20 @@
         <v>20</v>
       </c>
       <c r="H3" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="I3" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="J3" s="12" t="s">
         <v>34</v>
-      </c>
-      <c r="I3" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="J3" s="12" t="s">
-        <v>35</v>
       </c>
       <c r="K3" s="12"/>
       <c r="L3" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="M3" s="12" t="s">
         <v>37</v>
-      </c>
-      <c r="M3" s="12" t="s">
-        <v>38</v>
       </c>
       <c r="N3" s="12"/>
       <c r="O3" s="12"/>
@@ -829,7 +826,7 @@
     </row>
     <row r="4" spans="1:16">
       <c r="A4" s="8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B4" s="9">
         <v>3</v>
@@ -838,32 +835,32 @@
         <v>16</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E4" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="F4" s="9" t="s">
-        <v>24</v>
+      <c r="F4" s="9">
+        <v>2</v>
       </c>
       <c r="G4" s="9" t="s">
         <v>20</v>
       </c>
       <c r="H4" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="I4" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="J4" s="9" t="s">
         <v>34</v>
-      </c>
-      <c r="I4" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="J4" s="9" t="s">
-        <v>35</v>
       </c>
       <c r="K4" s="9"/>
       <c r="L4" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="M4" s="9" t="s">
         <v>40</v>
-      </c>
-      <c r="M4" s="9" t="s">
-        <v>41</v>
       </c>
       <c r="N4" s="9"/>
       <c r="O4" s="9"/>
@@ -871,7 +868,7 @@
     </row>
     <row r="5" spans="1:16">
       <c r="A5" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B5" s="12">
         <v>4</v>
@@ -880,7 +877,7 @@
         <v>16</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E5" s="12" t="s">
         <v>23</v>
@@ -894,14 +891,14 @@
       <c r="H5" s="12"/>
       <c r="I5" s="12"/>
       <c r="J5" s="12" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="K5" s="12"/>
       <c r="L5" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="M5" s="12" t="s">
         <v>42</v>
-      </c>
-      <c r="M5" s="12" t="s">
-        <v>43</v>
       </c>
       <c r="N5" s="12"/>
       <c r="O5" s="12"/>
@@ -909,7 +906,7 @@
     </row>
     <row r="6" spans="1:16">
       <c r="A6" s="8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B6" s="9">
         <v>5</v>
@@ -930,20 +927,20 @@
         <v>20</v>
       </c>
       <c r="H6" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="I6" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="J6" s="9" t="s">
         <v>34</v>
-      </c>
-      <c r="I6" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="J6" s="9" t="s">
-        <v>35</v>
       </c>
       <c r="K6" s="9"/>
       <c r="L6" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="M6" s="9" t="s">
         <v>44</v>
-      </c>
-      <c r="M6" s="9" t="s">
-        <v>45</v>
       </c>
       <c r="N6" s="9"/>
       <c r="O6" s="9"/>
@@ -951,7 +948,7 @@
     </row>
     <row r="7" spans="1:16">
       <c r="A7" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B7" s="3">
         <v>6</v>
@@ -965,25 +962,25 @@
       <c r="E7" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="F7" s="3" t="s">
-        <v>29</v>
+      <c r="F7" s="3">
+        <v>10</v>
       </c>
       <c r="G7" s="3" t="s">
         <v>20</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I7" s="3"/>
       <c r="J7" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="K7" s="3"/>
       <c r="L7" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N7" s="3"/>
       <c r="O7" s="3"/>
@@ -996,6 +993,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="cf35dce2-b600-471d-a6b0-9e8301b7851b">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="3de82841-ffbb-418b-a888-39c303bacd30" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101003EADB6AB950C774BBB9F1C75E500B284" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="101bf262c701ad3b79067f76f13f8957">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="cf35dce2-b600-471d-a6b0-9e8301b7851b" xmlns:ns3="3de82841-ffbb-418b-a888-39c303bacd30" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a75b904d2a00e23a3c27f0f1b23bc34b" ns2:_="" ns3:_="">
     <xsd:import namespace="cf35dce2-b600-471d-a6b0-9e8301b7851b"/>
@@ -1196,27 +1213,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="cf35dce2-b600-471d-a6b0-9e8301b7851b">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="3de82841-ffbb-418b-a888-39c303bacd30" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FE1093A5-D1C7-4298-AA6E-C83F607F0D93}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="cf35dce2-b600-471d-a6b0-9e8301b7851b"/>
+    <ds:schemaRef ds:uri="3de82841-ffbb-418b-a888-39c303bacd30"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D130B052-D1FC-457D-9411-92615ACD176E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A9E8B1E8-A15D-4BCB-B5A6-575EB6B71573}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1233,23 +1249,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FE1093A5-D1C7-4298-AA6E-C83F607F0D93}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="cf35dce2-b600-471d-a6b0-9e8301b7851b"/>
-    <ds:schemaRef ds:uri="3de82841-ffbb-418b-a888-39c303bacd30"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D130B052-D1FC-457D-9411-92615ACD176E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>